<commit_message>
Improvements: this way it works with voice messages on live
</commit_message>
<xml_diff>
--- a/TestsResults.xlsx
+++ b/TestsResults.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eric/Documents/Masters Degree/M10.-TFM/LUCIA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA78AD75-9296-8E47-A4FD-6E6E4F29ED02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5765FB6-499F-4F4F-B8E4-F3A51631199F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19740" xr2:uid="{F495DA44-20F5-FE41-B3AC-6342030998CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Users Tests" sheetId="1" r:id="rId1"/>
-    <sheet name="Objects Results" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1637" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1621" uniqueCount="108">
   <si>
     <t>Users</t>
   </si>
@@ -7866,336 +7865,4 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B48791D4-C270-814A-950A-B31B8F51264F}">
-  <dimension ref="A1:H33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="6" max="6" width="87.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="1"/>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A33" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>